<commit_message>
chore: publish carecommunication IG 5.0.2
</commit_message>
<xml_diff>
--- a/ig/carecommunication/StructureDefinition-medcom-careCommunication-communication.xlsx
+++ b/ig/carecommunication/StructureDefinition-medcom-careCommunication-communication.xlsx
@@ -33,7 +33,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>5.0.1</t>
+    <t>5.0.2</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-10-29T10:10:10+00:00</t>
+    <t>2026-02-13T11:55:29+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -2304,7 +2304,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="3" hidden="true">
+    <row r="3">
       <c r="A3" t="s" s="2">
         <v>84</v>
       </c>
@@ -2746,7 +2746,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="7" hidden="true">
+    <row r="7">
       <c r="A7" t="s" s="2">
         <v>113</v>
       </c>
@@ -3077,7 +3077,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="10" hidden="true">
+    <row r="10">
       <c r="A10" t="s" s="2">
         <v>138</v>
       </c>
@@ -3186,7 +3186,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="11" hidden="true">
+    <row r="11">
       <c r="A11" t="s" s="2">
         <v>146</v>
       </c>
@@ -3515,7 +3515,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="14" hidden="true">
+    <row r="14">
       <c r="A14" t="s" s="2">
         <v>164</v>
       </c>
@@ -3739,7 +3739,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="16" hidden="true">
+    <row r="16">
       <c r="A16" t="s" s="2">
         <v>175</v>
       </c>
@@ -4411,7 +4411,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="22" hidden="true">
+    <row r="22">
       <c r="A22" t="s" s="2">
         <v>213</v>
       </c>
@@ -5291,7 +5291,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="30" hidden="true">
+    <row r="30">
       <c r="A30" t="s" s="2">
         <v>260</v>
       </c>
@@ -5513,7 +5513,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="32" hidden="true">
+    <row r="32">
       <c r="A32" t="s" s="2">
         <v>278</v>
       </c>
@@ -5842,7 +5842,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="35" hidden="true">
+    <row r="35">
       <c r="A35" t="s" s="2">
         <v>286</v>
       </c>
@@ -6175,7 +6175,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="38" hidden="true">
+    <row r="38">
       <c r="A38" t="s" s="2">
         <v>296</v>
       </c>
@@ -6399,7 +6399,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="40" hidden="true">
+    <row r="40">
       <c r="A40" t="s" s="2">
         <v>309</v>
       </c>
@@ -6847,7 +6847,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="44" hidden="true">
+    <row r="44">
       <c r="A44" t="s" s="2">
         <v>336</v>
       </c>
@@ -7067,7 +7067,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="46" hidden="true">
+    <row r="46">
       <c r="A46" t="s" s="2">
         <v>348</v>
       </c>
@@ -7176,7 +7176,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="47" hidden="true">
+    <row r="47">
       <c r="A47" t="s" s="2">
         <v>355</v>
       </c>
@@ -7620,7 +7620,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="51" hidden="true">
+    <row r="51">
       <c r="A51" t="s" s="2">
         <v>365</v>
       </c>
@@ -7844,7 +7844,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="53" hidden="true">
+    <row r="53">
       <c r="A53" t="s" s="2">
         <v>370</v>
       </c>
@@ -8173,7 +8173,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="56" hidden="true">
+    <row r="56">
       <c r="A56" t="s" s="2">
         <v>386</v>
       </c>
@@ -9600,7 +9600,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="69" hidden="true">
+    <row r="69">
       <c r="A69" t="s" s="2">
         <v>447</v>
       </c>
@@ -9927,7 +9927,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="72" hidden="true">
+    <row r="72">
       <c r="A72" t="s" s="2">
         <v>453</v>
       </c>
@@ -10038,7 +10038,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="73" hidden="true">
+    <row r="73">
       <c r="A73" t="s" s="2">
         <v>454</v>
       </c>
@@ -10149,7 +10149,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="74" hidden="true">
+    <row r="74">
       <c r="A74" t="s" s="2">
         <v>455</v>
       </c>
@@ -10260,7 +10260,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="75" hidden="true">
+    <row r="75">
       <c r="A75" t="s" s="2">
         <v>456</v>
       </c>
@@ -10484,7 +10484,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="77" hidden="true">
+    <row r="77">
       <c r="A77" t="s" s="2">
         <v>458</v>
       </c>
@@ -10593,7 +10593,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="78" hidden="true">
+    <row r="78">
       <c r="A78" t="s" s="2">
         <v>460</v>
       </c>
@@ -10920,7 +10920,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="81" hidden="true">
+    <row r="81">
       <c r="A81" t="s" s="2">
         <v>466</v>
       </c>
@@ -11031,7 +11031,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="82" hidden="true">
+    <row r="82">
       <c r="A82" t="s" s="2">
         <v>467</v>
       </c>
@@ -11142,7 +11142,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="83" hidden="true">
+    <row r="83">
       <c r="A83" t="s" s="2">
         <v>468</v>
       </c>
@@ -11253,7 +11253,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="84" hidden="true">
+    <row r="84">
       <c r="A84" t="s" s="2">
         <v>469</v>
       </c>
@@ -11477,7 +11477,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="86" hidden="true">
+    <row r="86">
       <c r="A86" t="s" s="2">
         <v>471</v>
       </c>
@@ -11806,7 +11806,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="89" hidden="true">
+    <row r="89">
       <c r="A89" t="s" s="2">
         <v>477</v>
       </c>
@@ -12026,7 +12026,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="91" hidden="true">
+    <row r="91">
       <c r="A91" t="s" s="2">
         <v>494</v>
       </c>
@@ -12139,7 +12139,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="92" hidden="true">
+    <row r="92">
       <c r="A92" t="s" s="2">
         <v>503</v>
       </c>
@@ -12478,7 +12478,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="95" hidden="true">
+    <row r="95">
       <c r="A95" t="s" s="2">
         <v>530</v>
       </c>
@@ -12589,7 +12589,7 @@
         <v>537</v>
       </c>
     </row>
-    <row r="96" hidden="true">
+    <row r="96">
       <c r="A96" t="s" s="2">
         <v>538</v>
       </c>
@@ -12811,12 +12811,12 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:AM97">
-    <filterColumn colId="6">
+    <filterColumn colId="7">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
       </customFilters>
     </filterColumn>
-    <filterColumn colId="26">
+    <filterColumn colId="27">
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
chore: publish carecommunication IG 5.0.2 (#70)
Co-authored-by: olw-medcom <olw-medcom@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ig/carecommunication/StructureDefinition-medcom-careCommunication-communication.xlsx
+++ b/ig/carecommunication/StructureDefinition-medcom-careCommunication-communication.xlsx
@@ -33,7 +33,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>5.0.1</t>
+    <t>5.0.2</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-10-29T10:10:10+00:00</t>
+    <t>2026-02-13T11:55:29+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -2304,7 +2304,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="3" hidden="true">
+    <row r="3">
       <c r="A3" t="s" s="2">
         <v>84</v>
       </c>
@@ -2746,7 +2746,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="7" hidden="true">
+    <row r="7">
       <c r="A7" t="s" s="2">
         <v>113</v>
       </c>
@@ -3077,7 +3077,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="10" hidden="true">
+    <row r="10">
       <c r="A10" t="s" s="2">
         <v>138</v>
       </c>
@@ -3186,7 +3186,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="11" hidden="true">
+    <row r="11">
       <c r="A11" t="s" s="2">
         <v>146</v>
       </c>
@@ -3515,7 +3515,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="14" hidden="true">
+    <row r="14">
       <c r="A14" t="s" s="2">
         <v>164</v>
       </c>
@@ -3739,7 +3739,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="16" hidden="true">
+    <row r="16">
       <c r="A16" t="s" s="2">
         <v>175</v>
       </c>
@@ -4411,7 +4411,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="22" hidden="true">
+    <row r="22">
       <c r="A22" t="s" s="2">
         <v>213</v>
       </c>
@@ -5291,7 +5291,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="30" hidden="true">
+    <row r="30">
       <c r="A30" t="s" s="2">
         <v>260</v>
       </c>
@@ -5513,7 +5513,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="32" hidden="true">
+    <row r="32">
       <c r="A32" t="s" s="2">
         <v>278</v>
       </c>
@@ -5842,7 +5842,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="35" hidden="true">
+    <row r="35">
       <c r="A35" t="s" s="2">
         <v>286</v>
       </c>
@@ -6175,7 +6175,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="38" hidden="true">
+    <row r="38">
       <c r="A38" t="s" s="2">
         <v>296</v>
       </c>
@@ -6399,7 +6399,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="40" hidden="true">
+    <row r="40">
       <c r="A40" t="s" s="2">
         <v>309</v>
       </c>
@@ -6847,7 +6847,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="44" hidden="true">
+    <row r="44">
       <c r="A44" t="s" s="2">
         <v>336</v>
       </c>
@@ -7067,7 +7067,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="46" hidden="true">
+    <row r="46">
       <c r="A46" t="s" s="2">
         <v>348</v>
       </c>
@@ -7176,7 +7176,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="47" hidden="true">
+    <row r="47">
       <c r="A47" t="s" s="2">
         <v>355</v>
       </c>
@@ -7620,7 +7620,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="51" hidden="true">
+    <row r="51">
       <c r="A51" t="s" s="2">
         <v>365</v>
       </c>
@@ -7844,7 +7844,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="53" hidden="true">
+    <row r="53">
       <c r="A53" t="s" s="2">
         <v>370</v>
       </c>
@@ -8173,7 +8173,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="56" hidden="true">
+    <row r="56">
       <c r="A56" t="s" s="2">
         <v>386</v>
       </c>
@@ -9600,7 +9600,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="69" hidden="true">
+    <row r="69">
       <c r="A69" t="s" s="2">
         <v>447</v>
       </c>
@@ -9927,7 +9927,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="72" hidden="true">
+    <row r="72">
       <c r="A72" t="s" s="2">
         <v>453</v>
       </c>
@@ -10038,7 +10038,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="73" hidden="true">
+    <row r="73">
       <c r="A73" t="s" s="2">
         <v>454</v>
       </c>
@@ -10149,7 +10149,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="74" hidden="true">
+    <row r="74">
       <c r="A74" t="s" s="2">
         <v>455</v>
       </c>
@@ -10260,7 +10260,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="75" hidden="true">
+    <row r="75">
       <c r="A75" t="s" s="2">
         <v>456</v>
       </c>
@@ -10484,7 +10484,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="77" hidden="true">
+    <row r="77">
       <c r="A77" t="s" s="2">
         <v>458</v>
       </c>
@@ -10593,7 +10593,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="78" hidden="true">
+    <row r="78">
       <c r="A78" t="s" s="2">
         <v>460</v>
       </c>
@@ -10920,7 +10920,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="81" hidden="true">
+    <row r="81">
       <c r="A81" t="s" s="2">
         <v>466</v>
       </c>
@@ -11031,7 +11031,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="82" hidden="true">
+    <row r="82">
       <c r="A82" t="s" s="2">
         <v>467</v>
       </c>
@@ -11142,7 +11142,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="83" hidden="true">
+    <row r="83">
       <c r="A83" t="s" s="2">
         <v>468</v>
       </c>
@@ -11253,7 +11253,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="84" hidden="true">
+    <row r="84">
       <c r="A84" t="s" s="2">
         <v>469</v>
       </c>
@@ -11477,7 +11477,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="86" hidden="true">
+    <row r="86">
       <c r="A86" t="s" s="2">
         <v>471</v>
       </c>
@@ -11806,7 +11806,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="89" hidden="true">
+    <row r="89">
       <c r="A89" t="s" s="2">
         <v>477</v>
       </c>
@@ -12026,7 +12026,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="91" hidden="true">
+    <row r="91">
       <c r="A91" t="s" s="2">
         <v>494</v>
       </c>
@@ -12139,7 +12139,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="92" hidden="true">
+    <row r="92">
       <c r="A92" t="s" s="2">
         <v>503</v>
       </c>
@@ -12478,7 +12478,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="95" hidden="true">
+    <row r="95">
       <c r="A95" t="s" s="2">
         <v>530</v>
       </c>
@@ -12589,7 +12589,7 @@
         <v>537</v>
       </c>
     </row>
-    <row r="96" hidden="true">
+    <row r="96">
       <c r="A96" t="s" s="2">
         <v>538</v>
       </c>
@@ -12811,12 +12811,12 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:AM97">
-    <filterColumn colId="6">
+    <filterColumn colId="7">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
       </customFilters>
     </filterColumn>
-    <filterColumn colId="26">
+    <filterColumn colId="27">
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
chore: publish carecommunication IG 5.0.3
</commit_message>
<xml_diff>
--- a/ig/carecommunication/StructureDefinition-medcom-careCommunication-communication.xlsx
+++ b/ig/carecommunication/StructureDefinition-medcom-careCommunication-communication.xlsx
@@ -33,7 +33,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>5.0.2</t>
+    <t>5.0.3</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-02-13T11:55:29+00:00</t>
+    <t>2026-06-03T09:32:39+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
chore: publish carecommunication IG 5.0.3 (#82)
Co-authored-by: olw-medcom <olw-medcom@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ig/carecommunication/StructureDefinition-medcom-careCommunication-communication.xlsx
+++ b/ig/carecommunication/StructureDefinition-medcom-careCommunication-communication.xlsx
@@ -33,7 +33,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>5.0.2</t>
+    <t>5.0.3</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-02-13T11:55:29+00:00</t>
+    <t>2026-06-03T09:32:39+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
chore: publish carecommunication IG 5.0.4
</commit_message>
<xml_diff>
--- a/ig/carecommunication/StructureDefinition-medcom-careCommunication-communication.xlsx
+++ b/ig/carecommunication/StructureDefinition-medcom-careCommunication-communication.xlsx
@@ -33,7 +33,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>5.0.3</t>
+    <t>5.0.4</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-03T09:32:39+00:00</t>
+    <t>2026-06-05T08:11:03+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -263,7 +263,7 @@
   </si>
   <si>
     <t>dom-2:If the resource is contained in another resource, it SHALL NOT contain nested Resources {contained.contained.empty()}
-dom-3:If the resource is contained in another resource, it SHALL be referred to from elsewhere in the resource or SHALL refer to the containing resource {contained.where((('#'+id in (%resource.descendants().reference | %resource.descendants().as(canonical) | %resource.descendants().as(uri) | %resource.descendants().as(url))) or descendants().where(reference = '#').exists() or descendants().where(as(canonical) = '#').exists() or descendants().where(as(canonical) = '#').exists()).not()).trace('unmatched', id).empty()}dom-4:If a resource is contained in another resource, it SHALL NOT have a meta.versionId or a meta.lastUpdated {contained.meta.versionId.empty() and contained.meta.lastUpdated.empty()}dom-5:If a resource is contained in another resource, it SHALL NOT have a security label {contained.meta.security.empty()}dom-6:A resource should have narrative for robust management {text.`div`.exists()}medcom-careCommunication-5:Priority must not be present when Communication.category is other than 'regarding-referral' {where(category.coding.code != 'regarding-referral').priority.empty()}medcom-careCommunication-6:There shall exist a Communication.topic when Communication.category = 'other' {iif(category.coding.code != 'other', true, category.coding.code = 'other' and topic.exists())}medcom-careCommunication-7:There shall exist a practitioner role when using a PractitionerRole as author in a message segment. {payload.extension('http://medcomfhir.dk/ig/core/StructureDefinition/medcom-core-practitioner-extension').value.resolve().all(code.coding.code.exists() xor code.text.exists())}medcom-careCommunication-8:There shall exist a practitioner name when using a Practitioner as author in a message segment. {payload.where(extension('http://medcomfhir.dk/ig/core/StructureDefinition/medcom-core-practitioner-extension').exists()).extension.value.reference.resolve().practitioner.resolve().name.exists()}medcom-careCommunication-9:An episodeOfCare-identifier must be included when an Encounter instance is included. {iif(encounter.exists().not(), true, encounter.reference.resolve().episodeOfCare.identifier.exists())}medcom-careCommunication-15:If an Encounter resource is present in the bundle, there must be a reference to it in Communication.encounter. If no Encounter is present, Communication.encounter must not be populated. {iif(encounter.exists(), Communication.encounter.reference.exists(), Communication.encounter.exists().not())}</t>
+dom-3:If the resource is contained in another resource, it SHALL be referred to from elsewhere in the resource or SHALL refer to the containing resource {contained.where((('#'+id in (%resource.descendants().reference | %resource.descendants().as(canonical) | %resource.descendants().as(uri) | %resource.descendants().as(url))) or descendants().where(reference = '#').exists() or descendants().where(as(canonical) = '#').exists() or descendants().where(as(canonical) = '#').exists()).not()).trace('unmatched', id).empty()}dom-4:If a resource is contained in another resource, it SHALL NOT have a meta.versionId or a meta.lastUpdated {contained.meta.versionId.empty() and contained.meta.lastUpdated.empty()}dom-5:If a resource is contained in another resource, it SHALL NOT have a security label {contained.meta.security.empty()}dom-6:A resource should have narrative for robust management {text.`div`.exists()}medcom-careCommunication-5:Priority must not be present when Communication.category is other than 'regarding-referral' {where(category.coding.code != 'regarding-referral').priority.empty()}medcom-careCommunication-6:There shall exist a Communication.topic when Communication.category = 'other' {iif(category.coding.code != 'other', true, category.coding.code = 'other' and topic.exists())}medcom-careCommunication-7:There shall exist a practitioner role when using a PractitionerRole as author in a message segment. {payload.extension('http://medcomfhir.dk/ig/core/StructureDefinition/medcom-core-practitioner-extension').value.resolve().all(code.coding.code.exists() xor code.text.exists())}medcom-careCommunication-8:There shall exist a practitioner name when using a Practitioner as author in a message segment. {payload.where(extension('http://medcomfhir.dk/ig/core/StructureDefinition/medcom-core-practitioner-extension').exists()).extension.value.reference.resolve().practitioner.resolve().name.exists()}medcom-careCommunication-9:An episodeOfCare-identifier must be included when an Encounter instance is included. {iif(encounter.exists().not(), true, encounter.reference.resolve().episodeOfCare.identifier.exists())}</t>
   </si>
   <si>
     <t>Event</t>

</xml_diff>

<commit_message>
chore: publish carecommunication IG 5.0.4 (#84)
Co-authored-by: olw-medcom <olw-medcom@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ig/carecommunication/StructureDefinition-medcom-careCommunication-communication.xlsx
+++ b/ig/carecommunication/StructureDefinition-medcom-careCommunication-communication.xlsx
@@ -33,7 +33,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>5.0.3</t>
+    <t>5.0.4</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-03T09:32:39+00:00</t>
+    <t>2026-06-05T08:11:03+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -263,7 +263,7 @@
   </si>
   <si>
     <t>dom-2:If the resource is contained in another resource, it SHALL NOT contain nested Resources {contained.contained.empty()}
-dom-3:If the resource is contained in another resource, it SHALL be referred to from elsewhere in the resource or SHALL refer to the containing resource {contained.where((('#'+id in (%resource.descendants().reference | %resource.descendants().as(canonical) | %resource.descendants().as(uri) | %resource.descendants().as(url))) or descendants().where(reference = '#').exists() or descendants().where(as(canonical) = '#').exists() or descendants().where(as(canonical) = '#').exists()).not()).trace('unmatched', id).empty()}dom-4:If a resource is contained in another resource, it SHALL NOT have a meta.versionId or a meta.lastUpdated {contained.meta.versionId.empty() and contained.meta.lastUpdated.empty()}dom-5:If a resource is contained in another resource, it SHALL NOT have a security label {contained.meta.security.empty()}dom-6:A resource should have narrative for robust management {text.`div`.exists()}medcom-careCommunication-5:Priority must not be present when Communication.category is other than 'regarding-referral' {where(category.coding.code != 'regarding-referral').priority.empty()}medcom-careCommunication-6:There shall exist a Communication.topic when Communication.category = 'other' {iif(category.coding.code != 'other', true, category.coding.code = 'other' and topic.exists())}medcom-careCommunication-7:There shall exist a practitioner role when using a PractitionerRole as author in a message segment. {payload.extension('http://medcomfhir.dk/ig/core/StructureDefinition/medcom-core-practitioner-extension').value.resolve().all(code.coding.code.exists() xor code.text.exists())}medcom-careCommunication-8:There shall exist a practitioner name when using a Practitioner as author in a message segment. {payload.where(extension('http://medcomfhir.dk/ig/core/StructureDefinition/medcom-core-practitioner-extension').exists()).extension.value.reference.resolve().practitioner.resolve().name.exists()}medcom-careCommunication-9:An episodeOfCare-identifier must be included when an Encounter instance is included. {iif(encounter.exists().not(), true, encounter.reference.resolve().episodeOfCare.identifier.exists())}medcom-careCommunication-15:If an Encounter resource is present in the bundle, there must be a reference to it in Communication.encounter. If no Encounter is present, Communication.encounter must not be populated. {iif(encounter.exists(), Communication.encounter.reference.exists(), Communication.encounter.exists().not())}</t>
+dom-3:If the resource is contained in another resource, it SHALL be referred to from elsewhere in the resource or SHALL refer to the containing resource {contained.where((('#'+id in (%resource.descendants().reference | %resource.descendants().as(canonical) | %resource.descendants().as(uri) | %resource.descendants().as(url))) or descendants().where(reference = '#').exists() or descendants().where(as(canonical) = '#').exists() or descendants().where(as(canonical) = '#').exists()).not()).trace('unmatched', id).empty()}dom-4:If a resource is contained in another resource, it SHALL NOT have a meta.versionId or a meta.lastUpdated {contained.meta.versionId.empty() and contained.meta.lastUpdated.empty()}dom-5:If a resource is contained in another resource, it SHALL NOT have a security label {contained.meta.security.empty()}dom-6:A resource should have narrative for robust management {text.`div`.exists()}medcom-careCommunication-5:Priority must not be present when Communication.category is other than 'regarding-referral' {where(category.coding.code != 'regarding-referral').priority.empty()}medcom-careCommunication-6:There shall exist a Communication.topic when Communication.category = 'other' {iif(category.coding.code != 'other', true, category.coding.code = 'other' and topic.exists())}medcom-careCommunication-7:There shall exist a practitioner role when using a PractitionerRole as author in a message segment. {payload.extension('http://medcomfhir.dk/ig/core/StructureDefinition/medcom-core-practitioner-extension').value.resolve().all(code.coding.code.exists() xor code.text.exists())}medcom-careCommunication-8:There shall exist a practitioner name when using a Practitioner as author in a message segment. {payload.where(extension('http://medcomfhir.dk/ig/core/StructureDefinition/medcom-core-practitioner-extension').exists()).extension.value.reference.resolve().practitioner.resolve().name.exists()}medcom-careCommunication-9:An episodeOfCare-identifier must be included when an Encounter instance is included. {iif(encounter.exists().not(), true, encounter.reference.resolve().episodeOfCare.identifier.exists())}</t>
   </si>
   <si>
     <t>Event</t>

</xml_diff>